<commit_message>
Organize practice set by teacher category sets (10 study sets)
- Add Study Sets sheet to Excel with exact Ch.4/Ch.9 breakdown
- Practice Set columns: Study Set, In-Set # (e.g. 1 of 2)
- PDF reorganized with section dividers per category + formula sheet
- Fix HW crop when end anchor is on next page

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Exam Prep.xlsx
+++ b/Exam Prep.xlsx
@@ -1,18 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Study Plan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Question Bank" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Practice Set" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Answer Key" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Formula Sheet" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="By Category" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study Plan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study Sets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Question Bank" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Practice Set" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Answer Key" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formula Sheet" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Category" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -804,6 +805,285 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Set #</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Chapter</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Questions in Set</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Practice Q IDs</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Consumer Problems</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Q1, Q2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Labor-Leisure</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Q3, Q4</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Intertemporal Consumption</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Q5, Q6</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Elasticity / Types of Goods</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Q7, Q8, Q9</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Budget Line</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Q10</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Assumptions / Preferences</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Q11, Q12</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Insurance Problems</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Q13–Q17</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Risk Attitudes</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Q18–Q21</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Certainty Equivalent &amp; Risk Premium</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Q22, Q23</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Diversification</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Q24</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Ch.4 = 12 | Ch.9 = 12</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>24</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Q1–Q24</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1876,7 +2156,7 @@
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>MRS: ℓ/c = w → ℓ = 20(16−ℓ)+80 = 400−20ℓ → ℓ*=400/21≈19.05 → capped at 16? Recheck: ℓ = wL+V/w with L=16−ℓ → ℓ* = (w·16+V)/(2w) = (320+80)/40 = 10. ℓ*=10, L*=6, c*=200.</t>
+          <t>MRS: (β/α)(c/ℓ)=w → c=wℓ. Budget: wℓ=w(16−ℓ)+80 → ℓ*=(w·16+V)/(2w)=10. L*=6, c*=$200.</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
@@ -3480,1076 +3760,6 @@
           <t>Diversification reduces risk with negative correlation.</t>
         </is>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="25" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>Label</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>Chapter</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>Ref</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>Question</t>
-        </is>
-      </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
-        <is>
-          <t>Answer / Key</t>
-        </is>
-      </c>
-      <c r="J1" s="4" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>Consumer Problem #1</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>Consumer Problems</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>Homework 1 Ch.4</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>Ex 3.1–3.5</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr">
-        <is>
-          <t>Manuel: U(q1,q2) = 3q1^0.6 q2^0.4. Prices p1=5, p2=10, income=$100. Find q1*, q2*.</t>
-        </is>
-      </c>
-      <c r="H2" s="7" t="inlineStr">
-        <is>
-          <t>Multi-step</t>
-        </is>
-      </c>
-      <c r="I2" s="7" t="inlineStr"/>
-      <c r="J2" s="7" t="inlineStr">
-        <is>
-          <t>Full consumer theory problem.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>Consumer Problem #2</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>Consumer Problems</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>Sample Q Ch.4</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>Q26</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
-        <is>
-          <t>PA=$2, PB=$3, I=$120, U(A,B)=2A²B³. Write budget constraint, find optimal bundle, slopes at optimum.</t>
-        </is>
-      </c>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>Multi-step</t>
-        </is>
-      </c>
-      <c r="I3" s="7" t="inlineStr"/>
-      <c r="J3" s="7" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Labor-Leisure #1</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>Labor-Leisure</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>Course-style (not in uploads)</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>LL-1</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>Maria has 16 hours/day for leisure (ℓ) and work. Wage w=$20/hr, non-labor income V=$80. Utility U(c,ℓ)=c^0.5 ℓ^0.5 where c = w(16−ℓ)+V. Find optimal ℓ* and labor hours L*.</t>
-        </is>
-      </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>Multi-step</t>
-        </is>
-      </c>
-      <c r="I4" s="7" t="inlineStr"/>
-      <c r="J4" s="7" t="inlineStr">
-        <is>
-          <t>Standard labor-leisure Cobb-Douglas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Labor-Leisure #2</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>Labor-Leisure</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>Course-style (not in uploads)</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>LL-2</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>Same setup as LL-1 but wage rises to w=$30. Find new ℓ*, L*, c*. Does Maria work more or less?</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>Multi-step</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="inlineStr"/>
-      <c r="J5" s="7" t="inlineStr">
-        <is>
-          <t>Compare to LL-1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Intertemporal #1</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>Intertemporal Consumption</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>Sample Q Ch.4</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>Q41</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
-        <is>
-          <t>I1=10, I2=12, r=0.5, p1=p2=1, u(q1,q2)=q1·q2. Find q1*, q2*. Saving or borrowing?</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>Multi-step</t>
-        </is>
-      </c>
-      <c r="I6" s="7" t="inlineStr"/>
-      <c r="J6" s="7" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Intertemporal #2</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>Intertemporal Consumption</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>Mock Midterm 1</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>Q25</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>Using Q24 setup, optimal q1 in period 1?</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="I7" s="7" t="inlineStr"/>
-      <c r="J7" s="7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Elasticity #1</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>Elasticity / Types of Goods</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>Homework 1 Ch.4</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Ex 4.1–4.2</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
-          <t>Demand q=100−5p. Find Q at p=5 and p=10. Compute price elasticity at p=5.</t>
-        </is>
-      </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>Calc</t>
-        </is>
-      </c>
-      <c r="I8" s="7" t="inlineStr"/>
-      <c r="J8" s="7" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Elasticity #2</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>Elasticity / Types of Goods</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>Sample Q Ch.4</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>Q39</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>QA = 784 − 2PA − 3I − 4PO. At PA=2, I=100, PO=20: price, income, and cross-price elasticities.</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>Multi-step</t>
-        </is>
-      </c>
-      <c r="I9" s="7" t="inlineStr"/>
-      <c r="J9" s="7" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Elasticity #3</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>Elasticity / Types of Goods</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>Sample Q Ch.4</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>Q38</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>Apples &amp; bananas complements; apples inferior. Which demand function for apples?</t>
-        </is>
-      </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="I10" s="7" t="inlineStr"/>
-      <c r="J10" s="7" t="inlineStr">
-        <is>
-          <t>Negative on I (inferior), positive on PB (complement).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Budget Line</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>Budget Line</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>Sample Q Ch.4</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>Q10</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>Apples (horizontal), oranges (vertical). Price of apples rises $3→$6; price of oranges rises $2→$4. Budget line:</t>
-        </is>
-      </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="inlineStr"/>
-      <c r="J11" s="7" t="inlineStr">
-        <is>
-          <t>Slope unchanged (−PA/PO); income effectively halved.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Preferences #1</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>Assumptions / Preferences</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>Homework 1 Ch.4</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>Ex 2.2</t>
-        </is>
-      </c>
-      <c r="G12" s="7" t="inlineStr">
-        <is>
-          <t>Jackie goes to the movies. Movies: 'Avatar' and 'The Avengers.' She cannot decide which one to see. Does this violate any assumption on preferences?</t>
-        </is>
-      </c>
-      <c r="H12" s="7" t="inlineStr">
-        <is>
-          <t>Concept</t>
-        </is>
-      </c>
-      <c r="I12" s="7" t="inlineStr"/>
-      <c r="J12" s="7" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Preferences #2</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>Assumptions / Preferences</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>Sample Q Ch.4</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>Q8</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>Serena's IC is a straight line with slope −7/5 (X on horizontal). Which utility function represents her preferences? Options include u = X/5 + Y/7.</t>
-        </is>
-      </c>
-      <c r="H13" s="7" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="inlineStr"/>
-      <c r="J13" s="7" t="inlineStr">
-        <is>
-          <t>IC slope = MRS = (1/5)/(1/7) = 7/5.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Insurance #1</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>Insurance</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>Homework 2 Ch.9</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>Ex 3a</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>Tom: house $846,400, 25% chance $174,000 damage, u=√I. Max premium P for full insurance?</t>
-        </is>
-      </c>
-      <c r="H14" s="7" t="inlineStr">
-        <is>
-          <t>Calc</t>
-        </is>
-      </c>
-      <c r="I14" s="7" t="inlineStr"/>
-      <c r="J14" s="7" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Insurance #2</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>Insurance</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>Homework 2 Ch.9</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>Ex 3b</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
-        <is>
-          <t>Same Tom setup. Fair (actuarially fair) insurance premium?</t>
-        </is>
-      </c>
-      <c r="H15" s="7" t="inlineStr">
-        <is>
-          <t>Calc</t>
-        </is>
-      </c>
-      <c r="I15" s="7" t="inlineStr"/>
-      <c r="J15" s="7" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Insurance #3</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="D16" s="7" t="inlineStr">
-        <is>
-          <t>Insurance</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>Sample Q Ch.9</t>
-        </is>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>Q18</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="inlineStr">
-        <is>
-          <t>Sherman: Ferrari $230,900 + $50,000 cash. 25% chance $158,400 damage. u=√x. Max P and RP?</t>
-        </is>
-      </c>
-      <c r="H16" s="7" t="inlineStr">
-        <is>
-          <t>Multi-step</t>
-        </is>
-      </c>
-      <c r="I16" s="7" t="inlineStr"/>
-      <c r="J16" s="7" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Insurance #4</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>Insurance</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>Mock Midterm 1</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>Q27</t>
-        </is>
-      </c>
-      <c r="G17" s="7" t="inlineStr">
-        <is>
-          <t>$1,000 cash. 10% sick, doctor $500. Premium $100, copay $275 if sick. u=√I. E[u] with insurance?</t>
-        </is>
-      </c>
-      <c r="H17" s="7" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="I17" s="7" t="inlineStr"/>
-      <c r="J17" s="7" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>Insurance #5</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>Insurance</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>Mock Midterm 1</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>Q25–26</t>
-        </is>
-      </c>
-      <c r="G18" s="7" t="inlineStr">
-        <is>
-          <t>Car $10,000, 75% crash $3,600 damage. u=√I. Max P and RP?</t>
-        </is>
-      </c>
-      <c r="H18" s="7" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="I18" s="7" t="inlineStr"/>
-      <c r="J18" s="7" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>Risk Attitudes #1</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>Risk Attitudes</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>Homework 2 Ch.9</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>Ex 2</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="inlineStr">
-        <is>
-          <t>Mike's MU(I) graph given. Bet: pay $20 on dice 1–2, receive $10 on 3–6. Fair bet? Accept?</t>
-        </is>
-      </c>
-      <c r="H19" s="7" t="inlineStr">
-        <is>
-          <t>Concept</t>
-        </is>
-      </c>
-      <c r="I19" s="7" t="inlineStr"/>
-      <c r="J19" s="7" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>Risk Attitudes #2</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>Risk Attitudes</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>Sample Q Ch.9</t>
-        </is>
-      </c>
-      <c r="F20" s="7" t="inlineStr">
-        <is>
-          <t>Q6</t>
-        </is>
-      </c>
-      <c r="G20" s="7" t="inlineStr">
-        <is>
-          <t>Anna U(I)=I, Elsa U(I)=I^1.5. Anna is ___ and Elsa is ___.</t>
-        </is>
-      </c>
-      <c r="H20" s="7" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="I20" s="7" t="inlineStr"/>
-      <c r="J20" s="7" t="inlineStr">
-        <is>
-          <t>a&gt;1 → risk loving; a=1 → neutral; a&lt;1 → averse.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>Risk Attitudes #3</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>Risk Attitudes</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>Sample Q Ch.9</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>Q8</t>
-        </is>
-      </c>
-      <c r="G21" s="7" t="inlineStr">
-        <is>
-          <t>Graphs of u(I) for Marta and Hannah. Classify both.</t>
-        </is>
-      </c>
-      <c r="H21" s="7" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="I21" s="7" t="inlineStr"/>
-      <c r="J21" s="7" t="inlineStr">
-        <is>
-          <t>Concave vs convex utility.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="7" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>Risk Attitudes #4</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>Risk Attitudes</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>Mock Midterm 1</t>
-        </is>
-      </c>
-      <c r="F22" s="7" t="inlineStr">
-        <is>
-          <t>Q28</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr">
-        <is>
-          <t>Firmino bet: Reds win → friend pays $1; lose → Firmino pays $3. Mohamed U=I^0.7, Sadio U=I^2.3.</t>
-        </is>
-      </c>
-      <c r="H22" s="7" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="I22" s="7" t="inlineStr"/>
-      <c r="J22" s="7" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>Certainty Eq. &amp; RP #1</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>Certainty Equivalent &amp; Risk Premium</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>Homework 2 Ch.9</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>Ex 1</t>
-        </is>
-      </c>
-      <c r="G23" s="7" t="inlineStr">
-        <is>
-          <t>Investment: 80% → $200, 20% → $50. u(x)=√x. Find E[x], E[u], certainty equivalent, risk premium.</t>
-        </is>
-      </c>
-      <c r="H23" s="7" t="inlineStr">
-        <is>
-          <t>Multi-step</t>
-        </is>
-      </c>
-      <c r="I23" s="7" t="inlineStr"/>
-      <c r="J23" s="7" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>Certainty Eq. &amp; RP #2</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>Certainty Equivalent &amp; Risk Premium</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>Sample Q Ch.9</t>
-        </is>
-      </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>Q12</t>
-        </is>
-      </c>
-      <c r="G24" s="7" t="inlineStr">
-        <is>
-          <t>80% → $144, 20% → $81, u(x)=√x. Find E[u], E[x], CE, RP.</t>
-        </is>
-      </c>
-      <c r="H24" s="7" t="inlineStr">
-        <is>
-          <t>Multi-step</t>
-        </is>
-      </c>
-      <c r="I24" s="7" t="inlineStr"/>
-      <c r="J24" s="7" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>Diversification</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>Diversification</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>Sample Q Ch.9</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>Q22</t>
-        </is>
-      </c>
-      <c r="G25" s="7" t="inlineStr">
-        <is>
-          <t>Feng: companies A&amp;B (agriculture, positively correlated). Nan: C&amp;D (airline/oil, negatively correlated). Who has riskier portfolio?</t>
-        </is>
-      </c>
-      <c r="H25" s="7" t="inlineStr">
-        <is>
-          <t>Concept</t>
-        </is>
-      </c>
-      <c r="I25" s="7" t="inlineStr"/>
-      <c r="J25" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4557,6 +3767,1328 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Study Set</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>In-Set #</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Chapter</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Ref</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Answer / Key</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Set 1: Consumer Problems</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>1 of 2</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Consumer Problem #1</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>Consumer Problems</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>Homework 1 Ch.4</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Ex 3.1–3.5</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>Manuel: U(q1,q2) = 3q1^0.6 q2^0.4. Prices p1=5, p2=10, income=$100. Find q1*, q2*.</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>Multi-step</t>
+        </is>
+      </c>
+      <c r="K2" s="7" t="inlineStr"/>
+      <c r="L2" s="7" t="inlineStr">
+        <is>
+          <t>Full consumer theory problem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Set 1: Consumer Problems</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>2 of 2</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Consumer Problem #2</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Consumer Problems</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Sample Q Ch.4</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>Q26</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>PA=$2, PB=$3, I=$120, U(A,B)=2A²B³. Write budget constraint, find optimal bundle, slopes at optimum.</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>Multi-step</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr"/>
+      <c r="L3" s="7" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Set 2: Labor-Leisure</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>1 of 2</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Labor-Leisure #1</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Labor-Leisure</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Course-style (not in uploads)</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>LL-1</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>Maria has 16 hours/day for leisure (ℓ) and work. Wage w=$20/hr, non-labor income V=$80. Utility U(c,ℓ)=c^0.5 ℓ^0.5 where c = w(16−ℓ)+V. Find optimal ℓ* and labor hours L*.</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>Multi-step</t>
+        </is>
+      </c>
+      <c r="K4" s="7" t="inlineStr"/>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>Standard labor-leisure Cobb-Douglas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Set 2: Labor-Leisure</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>2 of 2</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Labor-Leisure #2</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Labor-Leisure</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Course-style (not in uploads)</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>LL-2</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>Same setup as LL-1 but wage rises to w=$30. Find new ℓ*, L*, c*. Does Maria work more or less?</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Multi-step</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr"/>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>Compare to LL-1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Set 3: Intertemporal Consumption</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>1 of 2</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Intertemporal #1</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>Intertemporal Consumption</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Sample Q Ch.4</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Q41</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>I1=10, I2=12, r=0.5, p1=p2=1, u(q1,q2)=q1·q2. Find q1*, q2*. Saving or borrowing?</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>Multi-step</t>
+        </is>
+      </c>
+      <c r="K6" s="7" t="inlineStr"/>
+      <c r="L6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Set 3: Intertemporal Consumption</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>2 of 2</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Intertemporal #2</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Intertemporal Consumption</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Mock Midterm 1</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Q25</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>Using Q24 setup, optimal q1 in period 1?</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>MC</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr"/>
+      <c r="L7" s="7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Set 4: Elasticity / Types of Goods</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>1 of 3</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Elasticity #1</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Elasticity / Types of Goods</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Homework 1 Ch.4</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Ex 4.1–4.2</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>Demand q=100−5p. Find Q at p=5 and p=10. Compute price elasticity at p=5.</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t>Calc</t>
+        </is>
+      </c>
+      <c r="K8" s="7" t="inlineStr"/>
+      <c r="L8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Set 4: Elasticity / Types of Goods</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>2 of 3</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Elasticity #2</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Elasticity / Types of Goods</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Sample Q Ch.4</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Q39</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>QA = 784 − 2PA − 3I − 4PO. At PA=2, I=100, PO=20: price, income, and cross-price elasticities.</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>Multi-step</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="inlineStr"/>
+      <c r="L9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Set 4: Elasticity / Types of Goods</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>3 of 3</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Elasticity #3</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Elasticity / Types of Goods</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>Sample Q Ch.4</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Q38</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>Apples &amp; bananas complements; apples inferior. Which demand function for apples?</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>MC</t>
+        </is>
+      </c>
+      <c r="K10" s="7" t="inlineStr"/>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>Negative on I (inferior), positive on PB (complement).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Set 5: Budget Line</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>1 of 1</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Budget Line</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Budget Line</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Sample Q Ch.4</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Q10</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>Apples (horizontal), oranges (vertical). Price of apples rises $3→$6; price of oranges rises $2→$4. Budget line:</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>MC</t>
+        </is>
+      </c>
+      <c r="K11" s="7" t="inlineStr"/>
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>Slope unchanged (−PA/PO); income effectively halved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Set 6: Assumptions / Preferences</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>1 of 2</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Preferences #1</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Assumptions / Preferences</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Homework 1 Ch.4</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Ex 2.2</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>Jackie goes to the movies. Movies: 'Avatar' and 'The Avengers.' She cannot decide which one to see. Does this violate any assumption on preferences?</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="inlineStr">
+        <is>
+          <t>Concept</t>
+        </is>
+      </c>
+      <c r="K12" s="7" t="inlineStr"/>
+      <c r="L12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Set 6: Assumptions / Preferences</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>2 of 2</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Preferences #2</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Assumptions / Preferences</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Sample Q Ch.4</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>Serena's IC is a straight line with slope −7/5 (X on horizontal). Which utility function represents her preferences? Options include u = X/5 + Y/7.</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>MC</t>
+        </is>
+      </c>
+      <c r="K13" s="7" t="inlineStr"/>
+      <c r="L13" s="7" t="inlineStr">
+        <is>
+          <t>IC slope = MRS = (1/5)/(1/7) = 7/5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Set 7: Insurance Problems</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>1 of 5</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Insurance #1</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Insurance</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>Homework 2 Ch.9</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Ex 3a</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>Tom: house $846,400, 25% chance $174,000 damage, u=√I. Max premium P for full insurance?</t>
+        </is>
+      </c>
+      <c r="J14" s="7" t="inlineStr">
+        <is>
+          <t>Calc</t>
+        </is>
+      </c>
+      <c r="K14" s="7" t="inlineStr"/>
+      <c r="L14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Set 7: Insurance Problems</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>2 of 5</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Insurance #2</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>Insurance</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Homework 2 Ch.9</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Ex 3b</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>Same Tom setup. Fair (actuarially fair) insurance premium?</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>Calc</t>
+        </is>
+      </c>
+      <c r="K15" s="7" t="inlineStr"/>
+      <c r="L15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Set 7: Insurance Problems</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>3 of 5</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Insurance #3</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Insurance</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Sample Q Ch.9</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Q18</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>Sherman: Ferrari $230,900 + $50,000 cash. 25% chance $158,400 damage. u=√x. Max P and RP?</t>
+        </is>
+      </c>
+      <c r="J16" s="7" t="inlineStr">
+        <is>
+          <t>Multi-step</t>
+        </is>
+      </c>
+      <c r="K16" s="7" t="inlineStr"/>
+      <c r="L16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Set 7: Insurance Problems</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>4 of 5</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Insurance #4</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Insurance</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Mock Midterm 1</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Q27</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>$1,000 cash. 10% sick, doctor $500. Premium $100, copay $275 if sick. u=√I. E[u] with insurance?</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>MC</t>
+        </is>
+      </c>
+      <c r="K17" s="7" t="inlineStr"/>
+      <c r="L17" s="7" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Set 7: Insurance Problems</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>5 of 5</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Insurance #5</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>Insurance</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Mock Midterm 1</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Q25–26</t>
+        </is>
+      </c>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>Car $10,000, 75% crash $3,600 damage. u=√I. Max P and RP?</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="inlineStr">
+        <is>
+          <t>MC</t>
+        </is>
+      </c>
+      <c r="K18" s="7" t="inlineStr"/>
+      <c r="L18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Set 8: Risk Attitudes</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>1 of 4</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Risk Attitudes #1</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>Risk Attitudes</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Homework 2 Ch.9</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Ex 2</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>Mike's MU(I) graph given. Bet: pay $20 on dice 1–2, receive $10 on 3–6. Fair bet? Accept?</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>Concept</t>
+        </is>
+      </c>
+      <c r="K19" s="7" t="inlineStr"/>
+      <c r="L19" s="7" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Set 8: Risk Attitudes</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>2 of 4</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Risk Attitudes #2</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>Risk Attitudes</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>Sample Q Ch.9</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="I20" s="7" t="inlineStr">
+        <is>
+          <t>Anna U(I)=I, Elsa U(I)=I^1.5. Anna is ___ and Elsa is ___.</t>
+        </is>
+      </c>
+      <c r="J20" s="7" t="inlineStr">
+        <is>
+          <t>MC</t>
+        </is>
+      </c>
+      <c r="K20" s="7" t="inlineStr"/>
+      <c r="L20" s="7" t="inlineStr">
+        <is>
+          <t>a&gt;1 → risk loving; a=1 → neutral; a&lt;1 → averse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Set 8: Risk Attitudes</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>3 of 4</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Risk Attitudes #3</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>Risk Attitudes</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>Sample Q Ch.9</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t>Graphs of u(I) for Marta and Hannah. Classify both.</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>MC</t>
+        </is>
+      </c>
+      <c r="K21" s="7" t="inlineStr"/>
+      <c r="L21" s="7" t="inlineStr">
+        <is>
+          <t>Concave vs convex utility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Set 8: Risk Attitudes</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>4 of 4</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Risk Attitudes #4</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>Risk Attitudes</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>Mock Midterm 1</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Q28</t>
+        </is>
+      </c>
+      <c r="I22" s="7" t="inlineStr">
+        <is>
+          <t>Firmino bet: Reds win → friend pays $1; lose → Firmino pays $3. Mohamed U=I^0.7, Sadio U=I^2.3.</t>
+        </is>
+      </c>
+      <c r="J22" s="7" t="inlineStr">
+        <is>
+          <t>MC</t>
+        </is>
+      </c>
+      <c r="K22" s="7" t="inlineStr"/>
+      <c r="L22" s="7" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Set 9: Certainty Equivalent &amp; Risk Premium</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>1 of 2</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Certainty Eq. &amp; RP #1</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Certainty Equivalent &amp; Risk Premium</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Homework 2 Ch.9</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Ex 1</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="inlineStr">
+        <is>
+          <t>Investment: 80% → $200, 20% → $50. u(x)=√x. Find E[x], E[u], certainty equivalent, risk premium.</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="inlineStr">
+        <is>
+          <t>Multi-step</t>
+        </is>
+      </c>
+      <c r="K23" s="7" t="inlineStr"/>
+      <c r="L23" s="7" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Set 9: Certainty Equivalent &amp; Risk Premium</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>2 of 2</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Certainty Eq. &amp; RP #2</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Certainty Equivalent &amp; Risk Premium</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Sample Q Ch.9</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Q12</t>
+        </is>
+      </c>
+      <c r="I24" s="7" t="inlineStr">
+        <is>
+          <t>80% → $144, 20% → $81, u(x)=√x. Find E[u], E[x], CE, RP.</t>
+        </is>
+      </c>
+      <c r="J24" s="7" t="inlineStr">
+        <is>
+          <t>Multi-step</t>
+        </is>
+      </c>
+      <c r="K24" s="7" t="inlineStr"/>
+      <c r="L24" s="7" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Set 10: Diversification</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>1 of 1</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Diversification</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Diversification</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>Sample Q Ch.9</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Q22</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="inlineStr">
+        <is>
+          <t>Feng: companies A&amp;B (agriculture, positively correlated). Nan: C&amp;D (airline/oil, negatively correlated). Who has riskier portfolio?</t>
+        </is>
+      </c>
+      <c r="J25" s="7" t="inlineStr">
+        <is>
+          <t>Concept</t>
+        </is>
+      </c>
+      <c r="K25" s="7" t="inlineStr"/>
+      <c r="L25" s="7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4649,7 +5181,7 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>MRS: ℓ/c = w → ℓ = 20(16−ℓ)+80 = 400−20ℓ → ℓ*=400/21≈19.05 → capped at 16? Recheck: ℓ = wL+V/w with L=16−ℓ → ℓ* = (w·16+V)/(2w) = (320+80)/40 = 10. ℓ*=10, L*=6, c*=200.</t>
+          <t>MRS: (β/α)(c/ℓ)=w → c=wℓ. Budget: wℓ=w(16−ℓ)+80 → ℓ*=(w·16+V)/(2w)=10. L*=6, c*=$200.</t>
         </is>
       </c>
     </row>
@@ -5078,7 +5610,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5569,7 +6101,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Split practice set into category PDFs with exact question counts
- 10 focused PDFs (one per topic) with teacher-specified counts
- Chapter 4/9 combined PDFs (12 Q each) and separate Formula_Sheet.pdf
- Practice_Sets.zip for one-click download
- Remove 64-page monolithic Exam_Prep.pdf
- Excel Study Sets sheet lists PDF filename per category

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Exam Prep.xlsx
+++ b/Exam Prep.xlsx
@@ -805,7 +805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -813,6 +813,7 @@
     <col width="36" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -841,6 +842,11 @@
           <t>Practice Q IDs</t>
         </is>
       </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>PDF File</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
@@ -862,6 +868,11 @@
           <t>Q1, Q2</t>
         </is>
       </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>01_Consumer_Problems.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
@@ -883,6 +894,11 @@
           <t>Q3, Q4</t>
         </is>
       </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>02_Labor_Leisure.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
@@ -904,6 +920,11 @@
           <t>Q5, Q6</t>
         </is>
       </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>03_Intertemporal_Consumption.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
@@ -925,6 +946,11 @@
           <t>Q7, Q8, Q9</t>
         </is>
       </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>04_Elasticity_Types_of_Goods.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
@@ -946,6 +972,11 @@
           <t>Q10</t>
         </is>
       </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>05_Budget_Line.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
@@ -967,6 +998,11 @@
           <t>Q11, Q12</t>
         </is>
       </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>06_Assumptions_Preferences.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">
@@ -988,6 +1024,11 @@
           <t>Q13–Q17</t>
         </is>
       </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>07_Insurance_Problems.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n">
@@ -1009,6 +1050,11 @@
           <t>Q18–Q21</t>
         </is>
       </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>08_Risk_Attitudes.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n">
@@ -1030,6 +1076,11 @@
           <t>Q22, Q23</t>
         </is>
       </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>09_Certainty_Equivalent_Risk_Premium.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n">
@@ -1051,6 +1102,11 @@
           <t>Q24</t>
         </is>
       </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>10_Diversification.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr"/>
@@ -1070,6 +1126,11 @@
       <c r="E12" t="inlineStr">
         <is>
           <t>Q1–Q24</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>practice_sets/ (10 PDFs + Formula_Sheet.pdf)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace category PDFs with full 24-question simulation practice tests
- 3 practice tests, each 24 Q in exact midterm format (Ch.4: 12, Ch.9: 12)
- Category counts per test: 2+2+2+3+1+2 and 5+4+2+1
- Different question combinations across tests from the 55-Q bank
- Separate Formula_Sheet.pdf (1 page)
- Practice_Tests.zip for one-click download

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Exam Prep.xlsx
+++ b/Exam Prep.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study Plan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study Sets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Question Bank" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Practice Set" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Answer Key" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formula Sheet" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Category" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exam Format" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Practice Tests" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Question Bank" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Practice Set" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Answer Key" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formula Sheet" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Category" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -787,7 +788,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>See 'Practice Set' sheet</t>
+          <t>See 'Practice Tests' sheet (3 full exams)</t>
         </is>
       </c>
     </row>
@@ -805,21 +806,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Set #</t>
+          <t>Section #</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
@@ -834,17 +834,12 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Questions in Set</t>
+          <t>Count</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Practice Q IDs</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>PDF File</t>
+          <t>Question #s on Test</t>
         </is>
       </c>
     </row>
@@ -865,12 +860,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>Q1, Q2</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>01_Consumer_Problems.pdf</t>
+          <t>Q1–Q2</t>
         </is>
       </c>
     </row>
@@ -891,12 +881,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Q3, Q4</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>02_Labor_Leisure.pdf</t>
+          <t>Q3–Q4</t>
         </is>
       </c>
     </row>
@@ -917,12 +902,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Q5, Q6</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>03_Intertemporal_Consumption.pdf</t>
+          <t>Q5–Q6</t>
         </is>
       </c>
     </row>
@@ -943,12 +923,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Q7, Q8, Q9</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>04_Elasticity_Types_of_Goods.pdf</t>
+          <t>Q7–Q9</t>
         </is>
       </c>
     </row>
@@ -972,11 +947,6 @@
           <t>Q10</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>05_Budget_Line.pdf</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
@@ -995,12 +965,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Q11, Q12</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>06_Assumptions_Preferences.pdf</t>
+          <t>Q11–Q12</t>
         </is>
       </c>
     </row>
@@ -1024,11 +989,6 @@
           <t>Q13–Q17</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>07_Insurance_Problems.pdf</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n">
@@ -1050,11 +1010,6 @@
           <t>Q18–Q21</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>08_Risk_Attitudes.pdf</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n">
@@ -1073,12 +1028,7 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Q22, Q23</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>09_Certainty_Equivalent_Risk_Premium.pdf</t>
+          <t>Q22–Q23</t>
         </is>
       </c>
     </row>
@@ -1102,17 +1052,11 @@
           <t>Q24</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>10_Diversification.pdf</t>
-        </is>
-      </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1125,12 +1069,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Q1–Q24</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>practice_sets/ (10 PDFs + Formula_Sheet.pdf)</t>
+          <t>Each practice test PDF has all 24</t>
         </is>
       </c>
     </row>
@@ -1140,6 +1079,102 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Test #</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>PDF File</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Total Q</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Bank IDs (in exam order)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Practice_Test_1.pdf</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Q014, Q015, Q021, Q022, Q025, Q027, Q028, Q032, Q031, Q008, Q002, Q005, Q047, Q048, Q050, Q052, Q053, Q039, Q040, Q042, Q045, Q035, Q036, Q054</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Practice_Test_2.pdf</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Q016, Q018, Q021, Q022, Q023, Q026, Q029, Q033, Q030, Q009, Q001, Q007, Q049, Q051, Q047, Q052, Q053, Q041, Q043, Q044, Q046, Q037, Q038, Q055</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Practice_Test_3.pdf</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Q017, Q019, Q021, Q022, Q024, Q027, Q028, Q034, Q032, Q010, Q003, Q004, Q048, Q050, Q049, Q051, Q053, Q039, Q041, Q042, Q046, Q035, Q037, Q054</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3827,7 +3862,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5149,7 +5184,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5671,7 +5706,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6162,7 +6197,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>